<commit_message>
excel banc de test jsp quoi
</commit_message>
<xml_diff>
--- a/Banc de tests/Mesures_Capteur_Graphite.xlsx
+++ b/Banc de tests/Mesures_Capteur_Graphite.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/050671fe9a2caa0f/Documents/INSA/4A/Capteurs/2024-2025-4GP-Clara-Anatolie/Banc de tests/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anato\OneDrive\Documents\INSA\4A\Capteur\Repositories\2024-2025-4GP-Clara-Anatolie\Banc de tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{B77437E2-7200-472B-8142-1DEDDEB09CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E291884B-2DD2-493C-A60D-628ED393D5BC}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{EB6AD448-40F3-403B-81CE-D21654A49612}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="4B tension" sheetId="1" r:id="rId1"/>
@@ -107,7 +106,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -308,7 +307,81 @@
             </c:spPr>
             <c:trendlineType val="linear"/>
             <c:dispRSqr val="0"/>
-            <c:dispEq val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="4.8844508752645233E-2"/>
+                  <c:y val="7.3675384875136224E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" sz="1050" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="accent1">
+                            <a:lumMod val="75000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                      </a:rPr>
+                      <a:t>y = 24,999x </a:t>
+                    </a:r>
+                    <a:endParaRPr lang="en-US" sz="1050">
+                      <a:solidFill>
+                        <a:schemeClr val="accent1">
+                          <a:lumMod val="75000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:endParaRPr>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
           </c:trendline>
           <c:xVal>
             <c:numRef>
@@ -411,7 +484,77 @@
             </c:spPr>
             <c:trendlineType val="linear"/>
             <c:dispRSqr val="0"/>
-            <c:dispEq val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="2.9851156425959577E-2"/>
+                  <c:y val="-6.6043882672560672E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="fr-FR" sz="1050" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="accent2"/>
+                        </a:solidFill>
+                      </a:rPr>
+                      <a:t>y = 27,158x </a:t>
+                    </a:r>
+                    <a:endParaRPr lang="fr-FR" sz="1050">
+                      <a:solidFill>
+                        <a:schemeClr val="accent2"/>
+                      </a:solidFill>
+                    </a:endParaRPr>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
           </c:trendline>
           <c:xVal>
             <c:numRef>
@@ -514,7 +657,69 @@
             </c:spPr>
             <c:trendlineType val="linear"/>
             <c:dispRSqr val="0"/>
-            <c:dispEq val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.1275470908016838E-4"/>
+                  <c:y val="-2.9725944344676215E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="fr-FR" sz="1050" baseline="0"/>
+                      <a:t>y = 48,551x </a:t>
+                    </a:r>
+                    <a:endParaRPr lang="fr-FR" sz="1050"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
           </c:trendline>
           <c:xVal>
             <c:numRef>
@@ -639,6 +844,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -761,6 +967,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -841,6 +1048,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -872,6 +1080,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -879,7 +1088,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -929,6 +1137,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1170,6 +1379,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1177,7 +1387,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1227,6 +1436,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1486,6 +1696,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1493,7 +1704,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1575,6 +1785,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1660,7 +1871,81 @@
             </c:spPr>
             <c:trendlineType val="linear"/>
             <c:dispRSqr val="0"/>
-            <c:dispEq val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.22561877553684012"/>
+                  <c:y val="-0.10437074725257343"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0">
+                        <a:ln>
+                          <a:solidFill>
+                            <a:schemeClr val="accent1"/>
+                          </a:solidFill>
+                        </a:ln>
+                      </a:rPr>
+                      <a:t>y = -11,619x </a:t>
+                    </a:r>
+                    <a:endParaRPr lang="en-US">
+                      <a:ln>
+                        <a:solidFill>
+                          <a:schemeClr val="accent1"/>
+                        </a:solidFill>
+                      </a:ln>
+                    </a:endParaRPr>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
           </c:trendline>
           <c:xVal>
             <c:numRef>
@@ -1751,7 +2036,81 @@
             </c:spPr>
             <c:trendlineType val="linear"/>
             <c:dispRSqr val="0"/>
-            <c:dispEq val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.28981662418834997"/>
+                  <c:y val="-0.20460260354362236"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="fr-FR" baseline="0">
+                        <a:ln>
+                          <a:solidFill>
+                            <a:schemeClr val="accent2"/>
+                          </a:solidFill>
+                        </a:ln>
+                      </a:rPr>
+                      <a:t>y = -15,749x </a:t>
+                    </a:r>
+                    <a:endParaRPr lang="fr-FR">
+                      <a:ln>
+                        <a:solidFill>
+                          <a:schemeClr val="accent2"/>
+                        </a:solidFill>
+                      </a:ln>
+                    </a:endParaRPr>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
           </c:trendline>
           <c:xVal>
             <c:numRef>
@@ -1854,7 +2213,69 @@
             </c:spPr>
             <c:trendlineType val="linear"/>
             <c:dispRSqr val="0"/>
-            <c:dispEq val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.25657332313370335"/>
+                  <c:y val="-0.21531516879296159"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="fr-FR" baseline="0"/>
+                      <a:t>y = -14,491x </a:t>
+                    </a:r>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
           </c:trendline>
           <c:xVal>
             <c:numRef>
@@ -1998,6 +2419,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -2127,6 +2549,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -2207,6 +2630,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2238,6 +2662,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2245,7 +2670,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2295,6 +2719,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2629,6 +3054,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2636,7 +3062,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2711,6 +3136,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3000,6 +3426,7 @@
         <c:idx val="2"/>
         <c:delete val="1"/>
       </c:legendEntry>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3031,6 +3458,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3038,7 +3466,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6536,14 +6963,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2150197</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>659914</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>72767</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>356932</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>390648</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>67901</xdr:rowOff>
     </xdr:to>
@@ -6951,7 +7378,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CF92F5E-7161-4D89-87DD-CF750AB5055C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -6994,11 +7421,11 @@
         <v>27209</v>
       </c>
       <c r="E2">
-        <f>D2-$D$2</f>
+        <f t="shared" ref="E2:E8" si="0">D2-$D$2</f>
         <v>0</v>
       </c>
       <c r="F2">
-        <f>E2/$D$2</f>
+        <f t="shared" ref="F2:F8" si="1">E2/$D$2</f>
         <v>0</v>
       </c>
     </row>
@@ -7016,11 +7443,11 @@
         <v>27338</v>
       </c>
       <c r="E3">
-        <f>D3-$D$2</f>
+        <f t="shared" si="0"/>
         <v>129</v>
       </c>
       <c r="F3">
-        <f>E3/$D$2</f>
+        <f t="shared" si="1"/>
         <v>4.7410783196736375E-3</v>
       </c>
     </row>
@@ -7038,11 +7465,11 @@
         <v>27449</v>
       </c>
       <c r="E4">
-        <f>D4-$D$2</f>
+        <f t="shared" si="0"/>
         <v>240</v>
       </c>
       <c r="F4">
-        <f>E4/$D$2</f>
+        <f t="shared" si="1"/>
         <v>8.8206108272997907E-3</v>
       </c>
     </row>
@@ -7060,11 +7487,11 @@
         <v>27894</v>
       </c>
       <c r="E5">
-        <f>D5-$D$2</f>
+        <f t="shared" si="0"/>
         <v>685</v>
       </c>
       <c r="F5">
-        <f>E5/$D$2</f>
+        <f t="shared" si="1"/>
         <v>2.517549340291815E-2</v>
       </c>
     </row>
@@ -7082,11 +7509,11 @@
         <v>28400</v>
       </c>
       <c r="E6">
-        <f>D6-$D$2</f>
+        <f t="shared" si="0"/>
         <v>1191</v>
       </c>
       <c r="F6">
-        <f>E6/$D$2</f>
+        <f t="shared" si="1"/>
         <v>4.3772281230475212E-2</v>
       </c>
     </row>
@@ -7104,11 +7531,11 @@
         <v>28700</v>
       </c>
       <c r="E7">
-        <f>D7-$D$2</f>
+        <f t="shared" si="0"/>
         <v>1491</v>
       </c>
       <c r="F7">
-        <f>E7/$D$2</f>
+        <f t="shared" si="1"/>
         <v>5.479804476459995E-2</v>
       </c>
     </row>
@@ -7126,11 +7553,11 @@
         <v>29050</v>
       </c>
       <c r="E8">
-        <f>D8-$D$2</f>
+        <f t="shared" si="0"/>
         <v>1841</v>
       </c>
       <c r="F8">
-        <f>E8/$D$2</f>
+        <f t="shared" si="1"/>
         <v>6.7661435554412147E-2</v>
       </c>
     </row>
@@ -7141,7 +7568,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C3BCE9-64D8-4C93-9C27-0CB4AD1314AB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7184,11 +7611,11 @@
         <v>117000</v>
       </c>
       <c r="E2">
-        <f>D2-$D$2</f>
+        <f t="shared" ref="E2:E8" si="0">D2-$D$2</f>
         <v>0</v>
       </c>
       <c r="F2">
-        <f>E2/$D$2</f>
+        <f t="shared" ref="F2:F8" si="1">E2/$D$2</f>
         <v>0</v>
       </c>
     </row>
@@ -7206,11 +7633,11 @@
         <v>123341</v>
       </c>
       <c r="E3">
-        <f>D3-$D$2</f>
+        <f t="shared" si="0"/>
         <v>6341</v>
       </c>
       <c r="F3">
-        <f>E3/$D$2</f>
+        <f t="shared" si="1"/>
         <v>5.4196581196581196E-2</v>
       </c>
     </row>
@@ -7228,11 +7655,11 @@
         <v>124672</v>
       </c>
       <c r="E4">
-        <f>D4-$D$2</f>
+        <f t="shared" si="0"/>
         <v>7672</v>
       </c>
       <c r="F4">
-        <f>E4/$D$2</f>
+        <f t="shared" si="1"/>
         <v>6.5572649572649577E-2</v>
       </c>
     </row>
@@ -7250,11 +7677,11 @@
         <v>125678</v>
       </c>
       <c r="E5">
-        <f>D5-$D$2</f>
+        <f t="shared" si="0"/>
         <v>8678</v>
       </c>
       <c r="F5">
-        <f>E5/$D$2</f>
+        <f t="shared" si="1"/>
         <v>7.4170940170940169E-2</v>
       </c>
     </row>
@@ -7272,11 +7699,11 @@
         <v>127400</v>
       </c>
       <c r="E6">
-        <f>D6-$D$2</f>
+        <f t="shared" si="0"/>
         <v>10400</v>
       </c>
       <c r="F6">
-        <f>E6/$D$2</f>
+        <f t="shared" si="1"/>
         <v>8.8888888888888892E-2</v>
       </c>
     </row>
@@ -7294,11 +7721,11 @@
         <v>128096</v>
       </c>
       <c r="E7">
-        <f>D7-$D$2</f>
+        <f t="shared" si="0"/>
         <v>11096</v>
       </c>
       <c r="F7">
-        <f>E7/$D$2</f>
+        <f t="shared" si="1"/>
         <v>9.4837606837606836E-2</v>
       </c>
     </row>
@@ -7316,11 +7743,11 @@
         <v>132320</v>
       </c>
       <c r="E8">
-        <f>D8-$D$2</f>
+        <f t="shared" si="0"/>
         <v>15320</v>
       </c>
       <c r="F8">
-        <f>E8/$D$2</f>
+        <f t="shared" si="1"/>
         <v>0.13094017094017094</v>
       </c>
     </row>
@@ -7331,7 +7758,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCF125B-5851-4C8E-A3AF-C4DCB05BA689}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7371,11 +7798,11 @@
         <v>186800</v>
       </c>
       <c r="E2">
-        <f>D2-$D$2</f>
+        <f t="shared" ref="E2:E7" si="0">D2-$D$2</f>
         <v>0</v>
       </c>
       <c r="F2">
-        <f>E2/$D$2</f>
+        <f t="shared" ref="F2:F7" si="1">E2/$D$2</f>
         <v>0</v>
       </c>
     </row>
@@ -7393,11 +7820,11 @@
         <v>210600</v>
       </c>
       <c r="E3">
-        <f>D3-$D$2</f>
+        <f t="shared" si="0"/>
         <v>23800</v>
       </c>
       <c r="F3">
-        <f>E3/$D$2</f>
+        <f t="shared" si="1"/>
         <v>0.12740899357601712</v>
       </c>
     </row>
@@ -7415,11 +7842,11 @@
         <v>214560</v>
       </c>
       <c r="E4">
-        <f>D4-$D$2</f>
+        <f t="shared" si="0"/>
         <v>27760</v>
       </c>
       <c r="F4">
-        <f>E4/$D$2</f>
+        <f t="shared" si="1"/>
         <v>0.14860813704496789</v>
       </c>
     </row>
@@ -7437,11 +7864,11 @@
         <v>219000</v>
       </c>
       <c r="E5">
-        <f>D5-$D$2</f>
+        <f t="shared" si="0"/>
         <v>32200</v>
       </c>
       <c r="F5">
-        <f>E5/$D$2</f>
+        <f t="shared" si="1"/>
         <v>0.17237687366167023</v>
       </c>
     </row>
@@ -7459,11 +7886,11 @@
         <v>223736</v>
       </c>
       <c r="E6">
-        <f>D6-$D$2</f>
+        <f t="shared" si="0"/>
         <v>36936</v>
       </c>
       <c r="F6">
-        <f>E6/$D$2</f>
+        <f t="shared" si="1"/>
         <v>0.19773019271948608</v>
       </c>
     </row>
@@ -7481,11 +7908,11 @@
         <v>234560</v>
       </c>
       <c r="E7">
-        <f>D7-$D$2</f>
+        <f t="shared" si="0"/>
         <v>47760</v>
       </c>
       <c r="F7">
-        <f>E7/$D$2</f>
+        <f t="shared" si="1"/>
         <v>0.25567451820128478</v>
       </c>
     </row>
@@ -7496,7 +7923,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBE14704-9C8A-4370-B3B7-9AB02F7FD6E1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7538,11 +7965,11 @@
         <v>48578</v>
       </c>
       <c r="E2">
-        <f>D2-$D$2</f>
+        <f t="shared" ref="E2:E8" si="0">D2-$D$2</f>
         <v>0</v>
       </c>
       <c r="F2">
-        <f>E2/$D$2</f>
+        <f t="shared" ref="F2:F8" si="1">E2/$D$2</f>
         <v>0</v>
       </c>
     </row>
@@ -7560,11 +7987,11 @@
         <v>48006</v>
       </c>
       <c r="E3">
-        <f>D3-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-572</v>
       </c>
       <c r="F3">
-        <f>E3/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-1.1774877516571287E-2</v>
       </c>
     </row>
@@ -7582,11 +8009,11 @@
         <v>47970</v>
       </c>
       <c r="E4">
-        <f>D4-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-608</v>
       </c>
       <c r="F4">
-        <f>E4/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-1.2515953723907942E-2</v>
       </c>
     </row>
@@ -7604,11 +8031,11 @@
         <v>47269</v>
       </c>
       <c r="E5" s="4">
-        <f>D5-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-1309</v>
       </c>
       <c r="F5" s="4">
-        <f>E5/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-2.6946354316768908E-2</v>
       </c>
     </row>
@@ -7626,11 +8053,11 @@
         <v>47400</v>
       </c>
       <c r="E6">
-        <f>D6-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-1178</v>
       </c>
       <c r="F6">
-        <f>E6/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-2.4249660340071637E-2</v>
       </c>
     </row>
@@ -7648,11 +8075,11 @@
         <v>47115</v>
       </c>
       <c r="E7">
-        <f>D7-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-1463</v>
       </c>
       <c r="F7">
-        <f>E7/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-3.0116513648153487E-2</v>
       </c>
     </row>
@@ -7670,11 +8097,11 @@
         <v>48387</v>
       </c>
       <c r="E8" s="4">
-        <f>D8-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-191</v>
       </c>
       <c r="F8" s="4">
-        <f>E8/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-3.9318209889250277E-3</v>
       </c>
     </row>
@@ -7685,7 +8112,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F1D1FAB-936E-4C77-8731-F3F5C599C03B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7727,11 +8154,11 @@
         <v>53444</v>
       </c>
       <c r="E2">
-        <f>D2-$D$2</f>
+        <f t="shared" ref="E2:E8" si="0">D2-$D$2</f>
         <v>0</v>
       </c>
       <c r="F2">
-        <f>E2/$D$2</f>
+        <f t="shared" ref="F2:F8" si="1">E2/$D$2</f>
         <v>0</v>
       </c>
     </row>
@@ -7749,11 +8176,11 @@
         <v>53024</v>
       </c>
       <c r="E3">
-        <f>D3-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-420</v>
       </c>
       <c r="F3">
-        <f>E3/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-7.8586932115859588E-3</v>
       </c>
     </row>
@@ -7771,11 +8198,11 @@
         <v>52870</v>
       </c>
       <c r="E4">
-        <f>D4-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-574</v>
       </c>
       <c r="F4">
-        <f>E4/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-1.0740214055834144E-2</v>
       </c>
     </row>
@@ -7793,11 +8220,11 @@
         <v>52340</v>
       </c>
       <c r="E5">
-        <f>D5-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-1104</v>
       </c>
       <c r="F5">
-        <f>E5/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-2.0657136441883092E-2</v>
       </c>
     </row>
@@ -7815,11 +8242,11 @@
         <v>51960</v>
       </c>
       <c r="E6">
-        <f>D6-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-1484</v>
       </c>
       <c r="F6">
-        <f>E6/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-2.7767382680937057E-2</v>
       </c>
     </row>
@@ -7837,11 +8264,11 @@
         <v>51573</v>
       </c>
       <c r="E7">
-        <f>D7-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-1871</v>
       </c>
       <c r="F7">
-        <f>E7/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-3.5008607140184118E-2</v>
       </c>
     </row>
@@ -7859,11 +8286,11 @@
         <v>50801</v>
       </c>
       <c r="E8">
-        <f>D8-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-2643</v>
       </c>
       <c r="F8">
-        <f>E8/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-4.9453633710051646E-2</v>
       </c>
     </row>
@@ -7874,7 +8301,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C954F671-BD54-4778-A3FA-5038C1C49DF3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7916,11 +8343,11 @@
         <v>585000</v>
       </c>
       <c r="E2">
-        <f>D2-$D$2</f>
+        <f t="shared" ref="E2:E8" si="0">D2-$D$2</f>
         <v>0</v>
       </c>
       <c r="F2">
-        <f>E2/$D$2</f>
+        <f t="shared" ref="F2:F8" si="1">E2/$D$2</f>
         <v>0</v>
       </c>
     </row>
@@ -7938,11 +8365,11 @@
         <v>575400</v>
       </c>
       <c r="E3">
-        <f>D3-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-9600</v>
       </c>
       <c r="F3">
-        <f>E3/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-1.641025641025641E-2</v>
       </c>
     </row>
@@ -7960,11 +8387,11 @@
         <v>566090</v>
       </c>
       <c r="E4">
-        <f>D4-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-18910</v>
       </c>
       <c r="F4">
-        <f>E4/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-3.2324786324786324E-2</v>
       </c>
     </row>
@@ -7982,11 +8409,11 @@
         <v>565408</v>
       </c>
       <c r="E5" s="4">
-        <f>D5-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-19592</v>
       </c>
       <c r="F5" s="4">
-        <f>E5/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-3.3490598290598292E-2</v>
       </c>
     </row>
@@ -8004,11 +8431,11 @@
         <v>564912</v>
       </c>
       <c r="E6">
-        <f>D6-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-20088</v>
       </c>
       <c r="F6">
-        <f>E6/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-3.433846153846154E-2</v>
       </c>
     </row>
@@ -8026,11 +8453,11 @@
         <v>561021</v>
       </c>
       <c r="E7" s="4">
-        <f>D7-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-23979</v>
       </c>
       <c r="F7" s="4">
-        <f>E7/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-4.0989743589743589E-2</v>
       </c>
     </row>
@@ -8048,11 +8475,11 @@
         <v>548294</v>
       </c>
       <c r="E8">
-        <f>D8-$D$2</f>
+        <f t="shared" si="0"/>
         <v>-36706</v>
       </c>
       <c r="F8">
-        <f>E8/$D$2</f>
+        <f t="shared" si="1"/>
         <v>-6.2745299145299152E-2</v>
       </c>
     </row>

</xml_diff>